<commit_message>
Finally got R package installed correctly (had to zip the folder first)
</commit_message>
<xml_diff>
--- a/Current Biodiversity Indicators.xlsx
+++ b/Current Biodiversity Indicators.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pbleefomgeving-my.sharepoint.com/personal/johnsonc_pbl_nl/Documents/Documents/Biodiversity data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pbleefomgeving-my.sharepoint.com/personal/johnsonc_pbl_nl/Documents/Documents/GLOBIO biodiversity data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="110" documentId="8_{84548B87-BBBE-447B-B1E9-8D6062FC6531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59CE81CC-A5F6-43A5-B599-C29B7C734F69}"/>
+  <xr:revisionPtr revIDLastSave="121" documentId="8_{84548B87-BBBE-447B-B1E9-8D6062FC6531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C04DDC42-FD45-4701-99B7-6ED81EBD8E96}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{37432F32-D47B-44E2-8C82-B935CA138876}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{37432F32-D47B-44E2-8C82-B935CA138876}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="25">
   <si>
     <t>Pressure</t>
   </si>
@@ -111,6 +111,9 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>Impact (slope)</t>
   </si>
 </sst>
 </file>
@@ -118,7 +121,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -157,12 +160,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -498,7 +507,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01E42F46-9383-48FB-88E4-7A45070772E4}">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.7109375" bestFit="1" customWidth="1"/>
@@ -510,123 +519,120 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="4"/>
+      <c r="D1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" s="4"/>
+      <c r="G1" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="5"/>
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="D2" s="5"/>
+      <c r="E2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="G2" s="5"/>
+      <c r="H2" s="1" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>0.46700000000000003</v>
-      </c>
-      <c r="C2">
-        <v>0.36199999999999999</v>
-      </c>
-      <c r="D2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>0.46700000000000003</v>
+      </c>
+      <c r="C3">
+        <v>0.36199999999999999</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="B3">
+      <c r="B4">
         <v>0.26400000000000001</v>
       </c>
-      <c r="C3">
+      <c r="C4">
         <v>0.36099999999999999</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D4" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E4" s="2">
         <f>1/(1+EXP(1.1))</f>
         <v>0.24973989440488234</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F4" s="2">
         <f>1/(1+EXP(1.15))</f>
         <v>0.24048908305088898</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>14</v>
       </c>
-      <c r="B4">
+      <c r="B5">
         <v>0.45200000000000001</v>
       </c>
-      <c r="C4">
+      <c r="C5">
         <v>0.156</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D5" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E5" s="2">
         <f>1/(1+EXP(1.44))</f>
         <v>0.19154534856146752</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F5" s="2">
         <f>1/(1+EXP(0.296))</f>
         <v>0.4265356063867507</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>0.40100000000000002</v>
-      </c>
-      <c r="C5">
-        <v>0.14899999999999999</v>
-      </c>
-      <c r="D5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B6">
-        <v>0.502</v>
+        <v>0.40100000000000002</v>
       </c>
       <c r="C6">
-        <v>0.16200000000000001</v>
+        <v>0.14899999999999999</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
@@ -636,54 +642,54 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="B7">
-        <v>0.45200000000000001</v>
+        <v>0.502</v>
       </c>
       <c r="C7">
-        <v>0.156</v>
+        <v>0.16200000000000001</v>
       </c>
       <c r="D7" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8">
+        <v>0.45200000000000001</v>
+      </c>
+      <c r="C8">
+        <v>0.156</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="2">
         <f>1/(1+EXP(1.11))</f>
         <v>0.2478708885604298</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F8" s="2">
         <f>1/(1+EXP(0.135))</f>
         <v>0.46630116456709919</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>0.40100000000000002</v>
-      </c>
-      <c r="C8">
-        <v>0.14899999999999999</v>
-      </c>
-      <c r="D8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9">
-        <v>0.502</v>
+        <v>0.40100000000000002</v>
       </c>
       <c r="C9">
-        <v>0.16200000000000001</v>
+        <v>0.14899999999999999</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
@@ -693,94 +699,117 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <v>0.502</v>
+      </c>
+      <c r="C10">
+        <v>0.16200000000000001</v>
+      </c>
+      <c r="D10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>9</v>
       </c>
-      <c r="B10">
+      <c r="B11">
         <v>0.58899999999999997</v>
       </c>
-      <c r="C10">
+      <c r="C11">
         <v>0.25900000000000001</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D11" t="s">
         <v>13</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E11" s="2">
         <f>1/(1+EXP(0.92))</f>
         <v>0.28495789429901025</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F11" s="2">
         <f>1/(1+EXP(-0.212))</f>
         <v>0.55280238544469373</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G11" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>0.621</v>
-      </c>
-      <c r="C11">
-        <v>0.56799999999999995</v>
-      </c>
-      <c r="D11" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <v>0.621</v>
+      </c>
+      <c r="C12">
+        <v>0.56799999999999995</v>
+      </c>
+      <c r="D12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B13" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C13" s="2">
         <f>1/(1+EXP(0.743))</f>
         <v>0.32234847500456443</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B14" s="2">
         <f>1/(1+EXP(1.39))</f>
         <v>0.19940775684866852</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D14" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B15" s="2">
         <f>1/(1+EXP(0.594))</f>
         <v>0.35571759580020623</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C15" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D15" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>20</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="G1:G2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>